<commit_message>
feat: unify industry hybrid retrieval and integrate report updates
</commit_message>
<xml_diff>
--- a/Creator Log/需求_记录文档.xlsx
+++ b/Creator Log/需求_记录文档.xlsx
@@ -3,8 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Postgraduate\科研\industry_graph-main\Creator Log\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28160" windowHeight="11040"/>
+    <workbookView windowHeight="17655"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
   <si>
     <t>产业洞察报告优化需求</t>
   </si>
@@ -897,8 +902,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8915400" y="5140960"/>
-          <a:ext cx="1386840" cy="424180"/>
+          <a:off x="10287000" y="4876800"/>
+          <a:ext cx="1569720" cy="449580"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -939,8 +944,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8915400" y="5928360"/>
-          <a:ext cx="1386840" cy="556260"/>
+          <a:off x="10287000" y="5715000"/>
+          <a:ext cx="1569720" cy="556260"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -981,8 +986,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8915400" y="7500620"/>
-          <a:ext cx="929640" cy="746760"/>
+          <a:off x="10287000" y="6762750"/>
+          <a:ext cx="1021080" cy="621030"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1255,15 +1260,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="5.33653846153846" customWidth="1"/>
-    <col min="2" max="2" width="70.1057692307692" customWidth="1"/>
-    <col min="3" max="3" width="50.5576923076923" customWidth="1"/>
-    <col min="7" max="7" width="16.2019230769231" customWidth="1"/>
+    <col min="1" max="1" width="5.33333333333333" customWidth="1"/>
+    <col min="2" max="2" width="70.1083333333333" customWidth="1"/>
+    <col min="3" max="3" width="50.5583333333333" customWidth="1"/>
+    <col min="7" max="7" width="16.2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" spans="1:7">
+    <row r="1" ht="21" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1273,7 +1278,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" ht="16.5" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1293,7 +1298,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" ht="16.5" spans="1:7">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -1314,7 +1319,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" ht="76" spans="1:7">
+    <row r="4" ht="66" spans="1:7">
       <c r="A4" s="6">
         <v>2</v>
       </c>
@@ -1332,7 +1337,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" ht="31" spans="1:7">
+    <row r="5" ht="33" spans="1:7">
       <c r="A5" s="6">
         <v>3</v>
       </c>
@@ -1348,7 +1353,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="31" spans="1:7">
+    <row r="6" ht="33" spans="1:7">
       <c r="A6" s="6">
         <v>4</v>
       </c>
@@ -1363,7 +1368,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" ht="92" spans="1:7">
+    <row r="7" ht="82.5" spans="1:7">
       <c r="A7" s="6">
         <v>5</v>
       </c>
@@ -1382,7 +1387,7 @@
       </c>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" ht="122" spans="1:7">
+    <row r="8" ht="115.5" spans="1:7">
       <c r="A8" s="6">
         <v>6</v>
       </c>
@@ -1401,7 +1406,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" ht="31" spans="1:7">
+    <row r="9" ht="33" spans="1:7">
       <c r="A9" s="6">
         <v>7</v>
       </c>
@@ -1415,9 +1420,11 @@
         <v>19</v>
       </c>
       <c r="E9" s="10"/>
-      <c r="F9" s="2"/>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="10" ht="31" spans="1:7">
+    <row r="10" ht="33" spans="1:7">
       <c r="A10" s="6">
         <v>8</v>
       </c>
@@ -1433,7 +1440,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" ht="107" spans="1:7">
+    <row r="11" ht="66" spans="1:7">
       <c r="A11" s="6">
         <v>9</v>
       </c>
@@ -1451,7 +1458,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" ht="16.5" spans="1:7">
       <c r="A12" s="6">
         <v>10</v>
       </c>
@@ -1482,7 +1489,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1494,7 +1501,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>